<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-19 16:40 UTC
</commit_message>
<xml_diff>
--- a/data/50001520 - XEMORTIZ DDG.xlsx
+++ b/data/50001520 - XEMORTIZ DDG.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="811" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="799" uniqueCount="233">
   <si>
     <t>50001520 -  XEMORTIZ DDG</t>
   </si>
@@ -151,7 +151,10 @@
     <t>Ingenieria Jefe de proyecto:</t>
   </si>
   <si>
-    <t>Ingenieria  Detalle,Ingenieria  Basica Motor,Ingenieria  basica Rodete,Analisis de costeo</t>
+    <t>Ingenieria  Detalle,Ingenieria  Basica Motor,Ingenieria  basica Rodete</t>
+  </si>
+  <si>
+    <t>Tarea en curso</t>
   </si>
   <si>
     <t>1213396196529409</t>
@@ -160,7 +163,7 @@
     <t>Ingenieria  Basica Motor</t>
   </si>
   <si>
-    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta motor</t>
+    <t>Ingenieria Jefe de proyecto:,propuesta motor</t>
   </si>
   <si>
     <t>1213396196529410</t>
@@ -169,7 +172,7 @@
     <t>Ingenieria  basica Rodete</t>
   </si>
   <si>
-    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta nucleo rodete,propuesta alabes</t>
+    <t>Ingenieria Jefe de proyecto:,propuesta nucleo rodete,propuesta alabes</t>
   </si>
   <si>
     <t>1213899724258045</t>
@@ -190,19 +193,7 @@
     <t>Ingenieria  Detalle</t>
   </si>
   <si>
-    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta compras a codigo // aprovisionamiento,Planos Preliminar</t>
-  </si>
-  <si>
-    <t>1213396196529412</t>
-  </si>
-  <si>
-    <t>Analisis de costeo</t>
-  </si>
-  <si>
-    <t>Ingenieria Jefe de proyecto:,Costos</t>
-  </si>
-  <si>
-    <t>Tarea en curso</t>
+    <t>Ingenieria Jefe de proyecto:,propuesta compras a codigo // aprovisionamiento,Planos Preliminar</t>
   </si>
   <si>
     <t>1213396196529413</t>
@@ -713,9 +704,6 @@
   </si>
   <si>
     <t>nicolas.tello@zitron.com</t>
-  </si>
-  <si>
-    <t>Despacho,Analisis de costeo</t>
   </si>
   <si>
     <t>1213458939855371</t>
@@ -1245,7 +1233,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U66"/>
+  <dimension ref="A1:U65"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10.4" customWidth="1"/>
@@ -1726,7 +1714,7 @@
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="5">
-        <v>46191.78179945602</v>
+        <v>46192.680794733795</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>45</v>
@@ -1762,11 +1750,13 @@
       <c r="R10" s="6"/>
       <c r="S10" s="6"/>
       <c r="T10" s="6"/>
-      <c r="U10" s="6"/>
+      <c r="U10" s="12" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B11" s="8">
         <v>46079.832187465276</v>
@@ -1775,10 +1765,10 @@
         <v>46097.54453039352</v>
       </c>
       <c r="D11" s="8">
-        <v>46097.54454956019</v>
+        <v>46192.680783703705</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>26</v>
@@ -1811,7 +1801,7 @@
         <v>40</v>
       </c>
       <c r="P11" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q11" s="8">
         <v>46084</v>
@@ -1831,7 +1821,7 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B12" s="5">
         <v>46079.832187754626</v>
@@ -1840,10 +1830,10 @@
         <v>46191.781787141204</v>
       </c>
       <c r="D12" s="5">
-        <v>46191.781807465275</v>
+        <v>46192.680783749995</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>26</v>
@@ -1876,7 +1866,7 @@
         <v>40</v>
       </c>
       <c r="P12" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q12" s="5">
         <v>46084</v>
@@ -1896,7 +1886,7 @@
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B13" s="8">
         <v>46114.51559517361</v>
@@ -1908,7 +1898,7 @@
         <v>46191.781849074076</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>26</v>
@@ -1935,7 +1925,7 @@
         <v>26</v>
       </c>
       <c r="N13" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="O13" s="9" t="s">
         <v>26</v>
@@ -1951,7 +1941,7 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B14" s="5">
         <v>46114.5157486574</v>
@@ -1963,7 +1953,7 @@
         <v>46191.781867453705</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>26</v>
@@ -1990,7 +1980,7 @@
         <v>26</v>
       </c>
       <c r="N14" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="O14" s="6" t="s">
         <v>26</v>
@@ -2006,7 +1996,7 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B15" s="8">
         <v>46079.83218810185</v>
@@ -2015,10 +2005,10 @@
         <v>46097.54473850694</v>
       </c>
       <c r="D15" s="8">
-        <v>46097.54475638889</v>
+        <v>46192.680783749995</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>26</v>
@@ -2051,7 +2041,7 @@
         <v>40</v>
       </c>
       <c r="P15" s="9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q15" s="8">
         <v>46084</v>
@@ -2071,33 +2061,29 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B16" s="5">
-        <v>46079.83218848379</v>
-      </c>
-      <c r="C16" s="6"/>
+        <v>46079.83218881945</v>
+      </c>
+      <c r="C16" s="5">
+        <v>46191.78195586806</v>
+      </c>
       <c r="D16" s="5">
-        <v>46191.78181219907</v>
+        <v>46191.781968599535</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="I16" s="5">
-        <v>46084</v>
-      </c>
-      <c r="J16" s="5">
-        <v>46087</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H16" s="6"/>
+      <c r="I16" s="6"/>
+      <c r="J16" s="6"/>
       <c r="K16" s="6" t="s">
         <v>26</v>
       </c>
@@ -2105,31 +2091,25 @@
         <v>26</v>
       </c>
       <c r="M16" s="6" t="s">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="N16" s="6" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="O16" s="6" t="s">
-        <v>41</v>
+        <v>63</v>
       </c>
       <c r="P16" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="Q16" s="5">
-        <v>46084</v>
-      </c>
-      <c r="R16" s="5">
-        <v>46087</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="Q16" s="6"/>
+      <c r="R16" s="6"/>
       <c r="S16" s="6">
-        <v>0</v>
-      </c>
-      <c r="T16" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="U16" s="12" t="s">
-        <v>63</v>
+        <v>1</v>
+      </c>
+      <c r="T16" s="6"/>
+      <c r="U16" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
@@ -2137,26 +2117,32 @@
         <v>64</v>
       </c>
       <c r="B17" s="8">
-        <v>46079.83218881945</v>
+        <v>46079.83218939815</v>
       </c>
       <c r="C17" s="8">
-        <v>46191.78195586806</v>
+        <v>46097.544778553245</v>
       </c>
       <c r="D17" s="8">
-        <v>46191.781968599535</v>
+        <v>46097.54544605324</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>65</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="9"/>
+        <v>35</v>
+      </c>
+      <c r="H17" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="I17" s="8">
+        <v>46086</v>
+      </c>
+      <c r="J17" s="8">
+        <v>46087</v>
+      </c>
       <c r="K17" s="9" t="s">
         <v>26</v>
       </c>
@@ -2164,23 +2150,29 @@
         <v>26</v>
       </c>
       <c r="M17" s="9" t="s">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="N17" s="9" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="O17" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="P17" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="P17" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q17" s="9"/>
-      <c r="R17" s="9"/>
+      <c r="Q17" s="8">
+        <v>46086</v>
+      </c>
+      <c r="R17" s="8">
+        <v>46087</v>
+      </c>
       <c r="S17" s="9">
         <v>1</v>
       </c>
-      <c r="T17" s="9"/>
+      <c r="T17" s="10" t="s">
+        <v>31</v>
+      </c>
       <c r="U17" s="11" t="s">
         <v>32</v>
       </c>
@@ -2190,13 +2182,13 @@
         <v>67</v>
       </c>
       <c r="B18" s="5">
-        <v>46079.83218939815</v>
+        <v>46079.83218971065</v>
       </c>
       <c r="C18" s="5">
-        <v>46097.544778553245</v>
+        <v>46191.781938229164</v>
       </c>
       <c r="D18" s="5">
-        <v>46097.54544605324</v>
+        <v>46191.78195724537</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>68</v>
@@ -2226,10 +2218,10 @@
         <v>26</v>
       </c>
       <c r="N18" s="6" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="P18" s="6" t="s">
         <v>69</v>
@@ -2255,13 +2247,13 @@
         <v>70</v>
       </c>
       <c r="B19" s="8">
-        <v>46079.83218971065</v>
+        <v>46079.8321903125</v>
       </c>
       <c r="C19" s="8">
-        <v>46191.781938229164</v>
+        <v>46191.78194402778</v>
       </c>
       <c r="D19" s="8">
-        <v>46191.78195724537</v>
+        <v>46191.781959687505</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>71</v>
@@ -2270,10 +2262,10 @@
         <v>26</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>35</v>
+        <v>72</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>36</v>
+        <v>72</v>
       </c>
       <c r="I19" s="8">
         <v>46086</v>
@@ -2291,13 +2283,13 @@
         <v>26</v>
       </c>
       <c r="N19" s="9" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="O19" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="P19" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q19" s="8">
         <v>46086</v>
@@ -2317,58 +2309,58 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B20" s="5">
-        <v>46079.8321903125</v>
+        <v>46079.83218699074</v>
       </c>
       <c r="C20" s="5">
-        <v>46191.78194402778</v>
+        <v>46097.54480537037</v>
       </c>
       <c r="D20" s="5">
-        <v>46191.781959687505</v>
+        <v>46100.77751619213</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="I20" s="5">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="J20" s="5">
+        <v>46090</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L20" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M20" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N20" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="O20" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="P20" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q20" s="5">
         <v>46087</v>
       </c>
-      <c r="K20" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L20" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M20" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N20" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="O20" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="P20" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="Q20" s="5">
-        <v>46086</v>
-      </c>
       <c r="R20" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="S20" s="6">
         <v>1</v>
@@ -2382,35 +2374,29 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B21" s="8">
-        <v>46079.83218699074</v>
+        <v>46079.83218734954</v>
       </c>
       <c r="C21" s="8">
-        <v>46097.54480537037</v>
+        <v>46192.68083542824</v>
       </c>
       <c r="D21" s="8">
-        <v>46100.77751619213</v>
+        <v>46192.680850335644</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="H21" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="I21" s="8">
-        <v>46087</v>
-      </c>
-      <c r="J21" s="8">
-        <v>46090</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9"/>
       <c r="K21" s="9" t="s">
         <v>26</v>
       </c>
@@ -2418,29 +2404,23 @@
         <v>26</v>
       </c>
       <c r="M21" s="9" t="s">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="N21" s="9" t="s">
-        <v>65</v>
+        <v>26</v>
       </c>
       <c r="O21" s="9" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="P21" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="Q21" s="8">
-        <v>46087</v>
-      </c>
-      <c r="R21" s="8">
-        <v>46090</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="Q21" s="9"/>
+      <c r="R21" s="9"/>
       <c r="S21" s="9">
         <v>1</v>
       </c>
-      <c r="T21" s="10" t="s">
-        <v>31</v>
-      </c>
+      <c r="T21" s="9"/>
       <c r="U21" s="11" t="s">
         <v>32</v>
       </c>
@@ -2450,24 +2430,32 @@
         <v>82</v>
       </c>
       <c r="B22" s="5">
-        <v>46079.83218734954</v>
-      </c>
-      <c r="C22" s="6"/>
+        <v>46079.832187673615</v>
+      </c>
+      <c r="C22" s="5">
+        <v>46191.782201967595</v>
+      </c>
       <c r="D22" s="5">
-        <v>46191.782222615744</v>
+        <v>46191.78221601852</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>83</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H22" s="6"/>
-      <c r="I22" s="6"/>
-      <c r="J22" s="6"/>
+        <v>84</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="I22" s="5">
+        <v>46090</v>
+      </c>
+      <c r="J22" s="5">
+        <v>46093</v>
+      </c>
       <c r="K22" s="6" t="s">
         <v>26</v>
       </c>
@@ -2475,55 +2463,63 @@
         <v>26</v>
       </c>
       <c r="M22" s="6" t="s">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="N22" s="6" t="s">
-        <v>26</v>
+        <v>80</v>
       </c>
       <c r="O22" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="P22" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q22" s="6"/>
-      <c r="R22" s="6"/>
-      <c r="S22" s="6"/>
-      <c r="T22" s="6"/>
-      <c r="U22" s="12" t="s">
-        <v>63</v>
+        <v>80</v>
+      </c>
+      <c r="Q22" s="5">
+        <v>46090</v>
+      </c>
+      <c r="R22" s="5">
+        <v>46093</v>
+      </c>
+      <c r="S22" s="6">
+        <v>1</v>
+      </c>
+      <c r="T22" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="U22" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B23" s="8">
+        <v>46079.83218790509</v>
+      </c>
+      <c r="C23" s="8">
+        <v>46191.78214869213</v>
+      </c>
+      <c r="D23" s="8">
+        <v>46191.78215086806</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G23" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="H23" s="9" t="s">
         <v>85</v>
-      </c>
-      <c r="B23" s="8">
-        <v>46079.832187673615</v>
-      </c>
-      <c r="C23" s="8">
-        <v>46191.782201967595</v>
-      </c>
-      <c r="D23" s="8">
-        <v>46191.78221601852</v>
-      </c>
-      <c r="E23" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G23" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="H23" s="9" t="s">
-        <v>88</v>
       </c>
       <c r="I23" s="8">
         <v>46090</v>
       </c>
       <c r="J23" s="8">
-        <v>46093</v>
+        <v>46091</v>
       </c>
       <c r="K23" s="9" t="s">
         <v>26</v>
@@ -2538,86 +2534,80 @@
         <v>83</v>
       </c>
       <c r="O23" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="P23" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="P23" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="Q23" s="8">
-        <v>46090</v>
-      </c>
-      <c r="R23" s="8">
-        <v>46093</v>
-      </c>
+      <c r="Q23" s="9"/>
+      <c r="R23" s="9"/>
       <c r="S23" s="9">
-        <v>1</v>
-      </c>
-      <c r="T23" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="U23" s="11" t="s">
-        <v>32</v>
+        <v>0</v>
+      </c>
+      <c r="T23" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="U23" s="10" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B24" s="5">
-        <v>46079.83218790509</v>
+        <v>46079.83218817129</v>
       </c>
       <c r="C24" s="5">
-        <v>46191.78214869213</v>
+        <v>46191.78218685185</v>
       </c>
       <c r="D24" s="5">
-        <v>46191.78215086806</v>
+        <v>46191.78218898148</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="H24" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="I24" s="5">
+        <v>46092</v>
+      </c>
+      <c r="J24" s="5">
+        <v>46093</v>
+      </c>
+      <c r="K24" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L24" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M24" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N24" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="O24" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="I24" s="5">
-        <v>46090</v>
-      </c>
-      <c r="J24" s="5">
-        <v>46091</v>
-      </c>
-      <c r="K24" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L24" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M24" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N24" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="O24" s="6" t="s">
-        <v>71</v>
-      </c>
       <c r="P24" s="6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="Q24" s="6"/>
       <c r="R24" s="6"/>
-      <c r="S24" s="6">
-        <v>0</v>
-      </c>
+      <c r="S24" s="6"/>
       <c r="T24" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="U24" s="10" t="s">
-        <v>94</v>
+        <v>90</v>
+      </c>
+      <c r="U24" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
@@ -2625,13 +2615,13 @@
         <v>95</v>
       </c>
       <c r="B25" s="8">
-        <v>46079.83218817129</v>
+        <v>46079.83218914352</v>
       </c>
       <c r="C25" s="8">
-        <v>46191.78218685185</v>
+        <v>46191.78212915509</v>
       </c>
       <c r="D25" s="8">
-        <v>46191.78218898148</v>
+        <v>46191.78214355324</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>96</v>
@@ -2640,16 +2630,16 @@
         <v>26</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="H25" s="9" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="I25" s="8">
-        <v>46092</v>
+        <v>46090</v>
       </c>
       <c r="J25" s="8">
-        <v>46093</v>
+        <v>46111</v>
       </c>
       <c r="K25" s="9" t="s">
         <v>26</v>
@@ -2661,19 +2651,25 @@
         <v>26</v>
       </c>
       <c r="N25" s="9" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="O25" s="9" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="P25" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="Q25" s="9"/>
-      <c r="R25" s="9"/>
-      <c r="S25" s="9"/>
-      <c r="T25" s="11" t="s">
-        <v>93</v>
+        <v>80</v>
+      </c>
+      <c r="Q25" s="8">
+        <v>46090</v>
+      </c>
+      <c r="R25" s="8">
+        <v>46111</v>
+      </c>
+      <c r="S25" s="9">
+        <v>1</v>
+      </c>
+      <c r="T25" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="U25" s="11" t="s">
         <v>32</v>
@@ -2684,13 +2680,13 @@
         <v>98</v>
       </c>
       <c r="B26" s="5">
-        <v>46079.83218914352</v>
+        <v>46079.832189374996</v>
       </c>
       <c r="C26" s="5">
-        <v>46191.78212915509</v>
+        <v>46191.782070057874</v>
       </c>
       <c r="D26" s="5">
-        <v>46191.78214355324</v>
+        <v>46191.78207137731</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>99</v>
@@ -2699,16 +2695,16 @@
         <v>26</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="I26" s="5">
         <v>46090</v>
       </c>
       <c r="J26" s="5">
-        <v>46111</v>
+        <v>46091</v>
       </c>
       <c r="K26" s="6" t="s">
         <v>26</v>
@@ -2720,28 +2716,24 @@
         <v>26</v>
       </c>
       <c r="N26" s="6" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="O26" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="P26" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="P26" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="Q26" s="5">
-        <v>46090</v>
-      </c>
-      <c r="R26" s="5">
-        <v>46111</v>
-      </c>
+      <c r="Q26" s="6"/>
+      <c r="R26" s="6"/>
       <c r="S26" s="6">
-        <v>1</v>
-      </c>
-      <c r="T26" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="U26" s="11" t="s">
-        <v>32</v>
+        <v>0</v>
+      </c>
+      <c r="T26" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="U26" s="10" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
@@ -2749,13 +2741,13 @@
         <v>101</v>
       </c>
       <c r="B27" s="8">
-        <v>46079.832189374996</v>
+        <v>46079.83218710648</v>
       </c>
       <c r="C27" s="8">
-        <v>46191.782070057874</v>
+        <v>46191.78211299768</v>
       </c>
       <c r="D27" s="8">
-        <v>46191.78207137731</v>
+        <v>46191.7821143287</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>102</v>
@@ -2764,16 +2756,16 @@
         <v>26</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="I27" s="8">
-        <v>46090</v>
+        <v>46092</v>
       </c>
       <c r="J27" s="8">
-        <v>46091</v>
+        <v>46111</v>
       </c>
       <c r="K27" s="9" t="s">
         <v>26</v>
@@ -2785,10 +2777,10 @@
         <v>26</v>
       </c>
       <c r="N27" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="O27" s="9" t="s">
         <v>99</v>
-      </c>
-      <c r="O27" s="9" t="s">
-        <v>74</v>
       </c>
       <c r="P27" s="9" t="s">
         <v>103</v>
@@ -2799,10 +2791,10 @@
         <v>0</v>
       </c>
       <c r="T27" s="11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="U27" s="10" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
@@ -2810,13 +2802,13 @@
         <v>104</v>
       </c>
       <c r="B28" s="5">
-        <v>46079.83218710648</v>
+        <v>46079.83218745371</v>
       </c>
       <c r="C28" s="5">
-        <v>46191.78211299768</v>
+        <v>46097.54557929398</v>
       </c>
       <c r="D28" s="5">
-        <v>46191.7821143287</v>
+        <v>46127.17852545139</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>105</v>
@@ -2825,16 +2817,16 @@
         <v>26</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="I28" s="5">
-        <v>46092</v>
+        <v>46090</v>
       </c>
       <c r="J28" s="5">
-        <v>46111</v>
+        <v>46126</v>
       </c>
       <c r="K28" s="6" t="s">
         <v>26</v>
@@ -2846,24 +2838,28 @@
         <v>26</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="P28" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="Q28" s="6"/>
-      <c r="R28" s="6"/>
+        <v>80</v>
+      </c>
+      <c r="Q28" s="5">
+        <v>46090</v>
+      </c>
+      <c r="R28" s="5">
+        <v>46126</v>
+      </c>
       <c r="S28" s="6">
-        <v>0</v>
-      </c>
-      <c r="T28" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="U28" s="10" t="s">
-        <v>94</v>
+        <v>1</v>
+      </c>
+      <c r="T28" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="U28" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
@@ -2871,13 +2867,13 @@
         <v>107</v>
       </c>
       <c r="B29" s="8">
-        <v>46079.83218745371</v>
+        <v>46079.83218777778</v>
       </c>
       <c r="C29" s="8">
-        <v>46097.54557929398</v>
+        <v>46097.545485752315</v>
       </c>
       <c r="D29" s="8">
-        <v>46127.17852545139</v>
+        <v>46097.54548765047</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>108</v>
@@ -2886,16 +2882,16 @@
         <v>26</v>
       </c>
       <c r="G29" s="9" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="H29" s="9" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="I29" s="8">
         <v>46090</v>
       </c>
       <c r="J29" s="8">
-        <v>46126</v>
+        <v>46098</v>
       </c>
       <c r="K29" s="9" t="s">
         <v>26</v>
@@ -2907,28 +2903,24 @@
         <v>26</v>
       </c>
       <c r="N29" s="9" t="s">
-        <v>83</v>
+        <v>105</v>
       </c>
       <c r="O29" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="P29" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="P29" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="Q29" s="8">
-        <v>46090</v>
-      </c>
-      <c r="R29" s="8">
-        <v>46126</v>
-      </c>
+      <c r="Q29" s="9"/>
+      <c r="R29" s="9"/>
       <c r="S29" s="9">
-        <v>1</v>
-      </c>
-      <c r="T29" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="U29" s="11" t="s">
-        <v>32</v>
+        <v>0</v>
+      </c>
+      <c r="T29" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="U29" s="10" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
@@ -2936,13 +2928,13 @@
         <v>110</v>
       </c>
       <c r="B30" s="5">
-        <v>46079.83218777778</v>
+        <v>46079.83218803241</v>
       </c>
       <c r="C30" s="5">
-        <v>46097.545485752315</v>
+        <v>46097.54553935185</v>
       </c>
       <c r="D30" s="5">
-        <v>46097.54548765047</v>
+        <v>46097.54554061343</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>111</v>
@@ -2951,16 +2943,16 @@
         <v>26</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="I30" s="5">
-        <v>46090</v>
+        <v>46099</v>
       </c>
       <c r="J30" s="5">
-        <v>46098</v>
+        <v>46126</v>
       </c>
       <c r="K30" s="6" t="s">
         <v>26</v>
@@ -2972,10 +2964,10 @@
         <v>26</v>
       </c>
       <c r="N30" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="O30" s="6" t="s">
         <v>108</v>
-      </c>
-      <c r="O30" s="6" t="s">
-        <v>68</v>
       </c>
       <c r="P30" s="6" t="s">
         <v>112</v>
@@ -2986,10 +2978,10 @@
         <v>0</v>
       </c>
       <c r="T30" s="11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="U30" s="10" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
@@ -2997,13 +2989,13 @@
         <v>113</v>
       </c>
       <c r="B31" s="8">
-        <v>46079.83218803241</v>
+        <v>46079.83218831019</v>
       </c>
       <c r="C31" s="8">
-        <v>46097.54553935185</v>
+        <v>46097.54556453704</v>
       </c>
       <c r="D31" s="8">
-        <v>46097.54554061343</v>
+        <v>46097.54556621528</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>114</v>
@@ -3012,16 +3004,16 @@
         <v>26</v>
       </c>
       <c r="G31" s="9" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="H31" s="9" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="I31" s="8">
         <v>46099</v>
       </c>
       <c r="J31" s="8">
-        <v>46126</v>
+        <v>46107</v>
       </c>
       <c r="K31" s="9" t="s">
         <v>26</v>
@@ -3033,10 +3025,10 @@
         <v>26</v>
       </c>
       <c r="N31" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="O31" s="9" t="s">
         <v>108</v>
-      </c>
-      <c r="O31" s="9" t="s">
-        <v>111</v>
       </c>
       <c r="P31" s="9" t="s">
         <v>115</v>
@@ -3047,10 +3039,10 @@
         <v>0</v>
       </c>
       <c r="T31" s="11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="U31" s="10" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
@@ -3058,13 +3050,13 @@
         <v>116</v>
       </c>
       <c r="B32" s="5">
-        <v>46079.83218831019</v>
+        <v>46079.83218859954</v>
       </c>
       <c r="C32" s="5">
-        <v>46097.54556453704</v>
+        <v>46112.505944282406</v>
       </c>
       <c r="D32" s="5">
-        <v>46097.54556621528</v>
+        <v>46120.17308952546</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>117</v>
@@ -3073,16 +3065,16 @@
         <v>26</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>87</v>
+        <v>118</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>88</v>
+        <v>119</v>
       </c>
       <c r="I32" s="5">
-        <v>46099</v>
+        <v>46091</v>
       </c>
       <c r="J32" s="5">
-        <v>46107</v>
+        <v>46119</v>
       </c>
       <c r="K32" s="6" t="s">
         <v>26</v>
@@ -3094,56 +3086,60 @@
         <v>26</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>108</v>
+        <v>80</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="P32" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="Q32" s="6"/>
-      <c r="R32" s="6"/>
+        <v>80</v>
+      </c>
+      <c r="Q32" s="5">
+        <v>46091</v>
+      </c>
+      <c r="R32" s="5">
+        <v>46119</v>
+      </c>
       <c r="S32" s="6">
-        <v>0</v>
-      </c>
-      <c r="T32" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="U32" s="10" t="s">
-        <v>94</v>
+        <v>1</v>
+      </c>
+      <c r="T32" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="U32" s="12" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="B33" s="8">
+        <v>46079.83218886574</v>
+      </c>
+      <c r="C33" s="8">
+        <v>46097.54567796296</v>
+      </c>
+      <c r="D33" s="8">
+        <v>46097.54567954861</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="F33" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G33" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="H33" s="9" t="s">
         <v>119</v>
-      </c>
-      <c r="B33" s="8">
-        <v>46079.83218859954</v>
-      </c>
-      <c r="C33" s="8">
-        <v>46112.505944282406</v>
-      </c>
-      <c r="D33" s="8">
-        <v>46120.17308952546</v>
-      </c>
-      <c r="E33" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="F33" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G33" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="H33" s="9" t="s">
-        <v>122</v>
       </c>
       <c r="I33" s="8">
         <v>46091</v>
       </c>
       <c r="J33" s="8">
-        <v>46119</v>
+        <v>46099</v>
       </c>
       <c r="K33" s="9" t="s">
         <v>26</v>
@@ -3155,28 +3151,24 @@
         <v>26</v>
       </c>
       <c r="N33" s="9" t="s">
-        <v>83</v>
+        <v>117</v>
       </c>
       <c r="O33" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="P33" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="P33" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="Q33" s="8">
-        <v>46091</v>
-      </c>
-      <c r="R33" s="8">
-        <v>46119</v>
-      </c>
+      <c r="Q33" s="9"/>
+      <c r="R33" s="9"/>
       <c r="S33" s="9">
-        <v>1</v>
-      </c>
-      <c r="T33" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="U33" s="12" t="s">
-        <v>63</v>
+        <v>0</v>
+      </c>
+      <c r="T33" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="U33" s="10" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
@@ -3184,13 +3176,13 @@
         <v>124</v>
       </c>
       <c r="B34" s="5">
-        <v>46079.83218886574</v>
+        <v>46079.83218913194</v>
       </c>
       <c r="C34" s="5">
-        <v>46097.54567796296</v>
+        <v>46112.50776791667</v>
       </c>
       <c r="D34" s="5">
-        <v>46097.54567954861</v>
+        <v>46112.50776931713</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>125</v>
@@ -3199,31 +3191,31 @@
         <v>26</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="H34" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="I34" s="5">
+        <v>46100</v>
+      </c>
+      <c r="J34" s="5">
+        <v>46119</v>
+      </c>
+      <c r="K34" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L34" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M34" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N34" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="O34" s="6" t="s">
         <v>122</v>
-      </c>
-      <c r="I34" s="5">
-        <v>46091</v>
-      </c>
-      <c r="J34" s="5">
-        <v>46099</v>
-      </c>
-      <c r="K34" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L34" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M34" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N34" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="O34" s="6" t="s">
-        <v>78</v>
       </c>
       <c r="P34" s="6" t="s">
         <v>126</v>
@@ -3234,10 +3226,10 @@
         <v>0</v>
       </c>
       <c r="T34" s="11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="U34" s="10" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
@@ -3245,32 +3237,24 @@
         <v>127</v>
       </c>
       <c r="B35" s="8">
-        <v>46079.83218913194</v>
-      </c>
-      <c r="C35" s="8">
-        <v>46112.50776791667</v>
-      </c>
+        <v>46079.83218939815</v>
+      </c>
+      <c r="C35" s="9"/>
       <c r="D35" s="8">
-        <v>46112.50776931713</v>
+        <v>46127.689880844904</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>128</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="H35" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="I35" s="8">
-        <v>46100</v>
-      </c>
-      <c r="J35" s="8">
-        <v>46119</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H35" s="9"/>
+      <c r="I35" s="9"/>
+      <c r="J35" s="9"/>
       <c r="K35" s="9" t="s">
         <v>26</v>
       </c>
@@ -3278,52 +3262,54 @@
         <v>26</v>
       </c>
       <c r="M35" s="9" t="s">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="N35" s="9" t="s">
-        <v>120</v>
+        <v>26</v>
       </c>
       <c r="O35" s="9" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="P35" s="9" t="s">
-        <v>129</v>
+        <v>26</v>
       </c>
       <c r="Q35" s="9"/>
       <c r="R35" s="9"/>
-      <c r="S35" s="9">
-        <v>0</v>
-      </c>
-      <c r="T35" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="U35" s="10" t="s">
-        <v>94</v>
-      </c>
+      <c r="S35" s="9"/>
+      <c r="T35" s="9"/>
+      <c r="U35" s="9"/>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
         <v>130</v>
       </c>
       <c r="B36" s="5">
-        <v>46079.83218939815</v>
-      </c>
-      <c r="C36" s="6"/>
+        <v>46079.83218966435</v>
+      </c>
+      <c r="C36" s="5">
+        <v>46114.51671186343</v>
+      </c>
       <c r="D36" s="5">
-        <v>46127.689880844904</v>
+        <v>46127.68903959491</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>131</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H36" s="6"/>
-      <c r="I36" s="6"/>
-      <c r="J36" s="6"/>
+        <v>132</v>
+      </c>
+      <c r="H36" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="I36" s="5">
+        <v>46087</v>
+      </c>
+      <c r="J36" s="5">
+        <v>46093</v>
+      </c>
       <c r="K36" s="6" t="s">
         <v>26</v>
       </c>
@@ -3331,53 +3317,63 @@
         <v>26</v>
       </c>
       <c r="M36" s="6" t="s">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="N36" s="6" t="s">
-        <v>26</v>
+        <v>128</v>
       </c>
       <c r="O36" s="6" t="s">
-        <v>132</v>
+        <v>59</v>
       </c>
       <c r="P36" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q36" s="6"/>
-      <c r="R36" s="6"/>
-      <c r="S36" s="6"/>
-      <c r="T36" s="6"/>
-      <c r="U36" s="6"/>
+        <v>134</v>
+      </c>
+      <c r="Q36" s="5">
+        <v>46087</v>
+      </c>
+      <c r="R36" s="5">
+        <v>46093</v>
+      </c>
+      <c r="S36" s="6">
+        <v>1</v>
+      </c>
+      <c r="T36" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="U36" s="11" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="B37" s="8">
+        <v>46079.832188009255</v>
+      </c>
+      <c r="C37" s="8">
+        <v>46127.68911905093</v>
+      </c>
+      <c r="D37" s="8">
+        <v>46127.689135925924</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="F37" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G37" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="H37" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="B37" s="8">
-        <v>46079.83218966435</v>
-      </c>
-      <c r="C37" s="8">
-        <v>46114.51671186343</v>
-      </c>
-      <c r="D37" s="8">
-        <v>46127.68903959491</v>
-      </c>
-      <c r="E37" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="F37" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G37" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="H37" s="9" t="s">
-        <v>136</v>
-      </c>
       <c r="I37" s="8">
-        <v>46087</v>
+        <v>46108</v>
       </c>
       <c r="J37" s="8">
-        <v>46093</v>
+        <v>46114</v>
       </c>
       <c r="K37" s="9" t="s">
         <v>26</v>
@@ -3389,19 +3385,19 @@
         <v>26</v>
       </c>
       <c r="N37" s="9" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="O37" s="9" t="s">
-        <v>58</v>
+        <v>137</v>
       </c>
       <c r="P37" s="9" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="Q37" s="8">
-        <v>46087</v>
+        <v>46108</v>
       </c>
       <c r="R37" s="8">
-        <v>46093</v>
+        <v>46114</v>
       </c>
       <c r="S37" s="9">
         <v>1</v>
@@ -3415,58 +3411,58 @@
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B38" s="5">
-        <v>46079.832188009255</v>
+        <v>46087.77438462963</v>
       </c>
       <c r="C38" s="5">
-        <v>46127.68911905093</v>
+        <v>46127.689870625</v>
       </c>
       <c r="D38" s="5">
-        <v>46127.689135925924</v>
+        <v>46127.68990261574</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="H38" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="I38" s="5">
+        <v>46115</v>
+      </c>
+      <c r="J38" s="5">
+        <v>46115</v>
+      </c>
+      <c r="K38" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L38" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M38" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N38" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="O38" s="6" t="s">
         <v>136</v>
-      </c>
-      <c r="I38" s="5">
-        <v>46108</v>
-      </c>
-      <c r="J38" s="5">
-        <v>46114</v>
-      </c>
-      <c r="K38" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L38" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M38" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N38" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="O38" s="6" t="s">
-        <v>140</v>
       </c>
       <c r="P38" s="6" t="s">
         <v>141</v>
       </c>
       <c r="Q38" s="5">
-        <v>46108</v>
+        <v>46115</v>
       </c>
       <c r="R38" s="5">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="S38" s="6">
         <v>1</v>
@@ -3483,13 +3479,11 @@
         <v>142</v>
       </c>
       <c r="B39" s="8">
-        <v>46087.77438462963</v>
-      </c>
-      <c r="C39" s="8">
-        <v>46127.689870625</v>
-      </c>
+        <v>46087.77498508102</v>
+      </c>
+      <c r="C39" s="9"/>
       <c r="D39" s="8">
-        <v>46127.68990261574</v>
+        <v>46150.16914774306</v>
       </c>
       <c r="E39" s="9" t="s">
         <v>143</v>
@@ -3498,16 +3492,14 @@
         <v>26</v>
       </c>
       <c r="G39" s="9" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="H39" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="I39" s="8">
-        <v>46115</v>
-      </c>
+        <v>145</v>
+      </c>
+      <c r="I39" s="9"/>
       <c r="J39" s="8">
-        <v>46115</v>
+        <v>46150</v>
       </c>
       <c r="K39" s="9" t="s">
         <v>26</v>
@@ -3519,57 +3511,55 @@
         <v>26</v>
       </c>
       <c r="N39" s="9" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="O39" s="9" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="P39" s="9" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="Q39" s="8">
-        <v>46115</v>
+        <v>46150</v>
       </c>
       <c r="R39" s="8">
-        <v>46115</v>
+        <v>46150</v>
       </c>
       <c r="S39" s="9">
-        <v>1</v>
-      </c>
-      <c r="T39" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="U39" s="11" t="s">
-        <v>32</v>
+        <v>0</v>
+      </c>
+      <c r="T39" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="U39" s="10" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B40" s="5">
-        <v>46087.77498508102</v>
-      </c>
-      <c r="C40" s="6"/>
+        <v>46079.83218837963</v>
+      </c>
+      <c r="C40" s="5">
+        <v>46191.78224238426</v>
+      </c>
       <c r="D40" s="5">
-        <v>46150.16914774306</v>
+        <v>46191.78225478009</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="H40" s="6" t="s">
-        <v>148</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H40" s="6"/>
       <c r="I40" s="6"/>
-      <c r="J40" s="5">
-        <v>46150</v>
-      </c>
+      <c r="J40" s="6"/>
       <c r="K40" s="6" t="s">
         <v>26</v>
       </c>
@@ -3577,31 +3567,25 @@
         <v>26</v>
       </c>
       <c r="M40" s="6" t="s">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>131</v>
+        <v>26</v>
       </c>
       <c r="O40" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="P40" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="Q40" s="5">
-        <v>46150</v>
-      </c>
-      <c r="R40" s="5">
-        <v>46150</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="Q40" s="6"/>
+      <c r="R40" s="6"/>
       <c r="S40" s="6">
-        <v>0</v>
-      </c>
-      <c r="T40" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="U40" s="10" t="s">
-        <v>94</v>
+        <v>1</v>
+      </c>
+      <c r="T40" s="6"/>
+      <c r="U40" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
@@ -3609,26 +3593,32 @@
         <v>151</v>
       </c>
       <c r="B41" s="8">
-        <v>46079.83218837963</v>
+        <v>46079.83218865741</v>
       </c>
       <c r="C41" s="8">
-        <v>46191.78224238426</v>
+        <v>46191.78222800926</v>
       </c>
       <c r="D41" s="8">
-        <v>46191.78225478009</v>
+        <v>46191.78224288195</v>
       </c>
       <c r="E41" s="9" t="s">
         <v>152</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G41" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H41" s="9"/>
-      <c r="I41" s="9"/>
-      <c r="J41" s="9"/>
+        <v>153</v>
+      </c>
+      <c r="H41" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="I41" s="8">
+        <v>46120</v>
+      </c>
+      <c r="J41" s="8">
+        <v>46121</v>
+      </c>
       <c r="K41" s="9" t="s">
         <v>26</v>
       </c>
@@ -3636,57 +3626,63 @@
         <v>26</v>
       </c>
       <c r="M41" s="9" t="s">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="N41" s="9" t="s">
-        <v>26</v>
+        <v>149</v>
       </c>
       <c r="O41" s="9" t="s">
-        <v>153</v>
+        <v>125</v>
       </c>
       <c r="P41" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q41" s="9"/>
-      <c r="R41" s="9"/>
+        <v>155</v>
+      </c>
+      <c r="Q41" s="8">
+        <v>46120</v>
+      </c>
+      <c r="R41" s="8">
+        <v>46121</v>
+      </c>
       <c r="S41" s="9">
         <v>1</v>
       </c>
-      <c r="T41" s="9"/>
+      <c r="T41" s="10" t="s">
+        <v>31</v>
+      </c>
       <c r="U41" s="11" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B42" s="5">
-        <v>46079.83218865741</v>
+        <v>46079.83218892361</v>
       </c>
       <c r="C42" s="5">
-        <v>46191.78222800926</v>
+        <v>46191.781853368055</v>
       </c>
       <c r="D42" s="5">
-        <v>46191.78224288195</v>
+        <v>46191.78224165509</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F42" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="I42" s="5">
-        <v>46120</v>
+        <v>46122</v>
       </c>
       <c r="J42" s="5">
-        <v>46121</v>
+        <v>46125</v>
       </c>
       <c r="K42" s="6" t="s">
         <v>26</v>
@@ -3698,19 +3694,19 @@
         <v>26</v>
       </c>
       <c r="N42" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="O42" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="O42" s="6" t="s">
-        <v>128</v>
-      </c>
       <c r="P42" s="6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="Q42" s="5">
-        <v>46120</v>
+        <v>46122</v>
       </c>
       <c r="R42" s="5">
-        <v>46121</v>
+        <v>46125</v>
       </c>
       <c r="S42" s="6">
         <v>1</v>
@@ -3718,41 +3714,35 @@
       <c r="T42" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U42" s="11" t="s">
-        <v>32</v>
+      <c r="U42" s="12" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B43" s="8">
-        <v>46079.83218892361</v>
+        <v>46079.83218921296</v>
       </c>
       <c r="C43" s="8">
-        <v>46191.781853368055</v>
+        <v>46191.78230420139</v>
       </c>
       <c r="D43" s="8">
-        <v>46191.78224165509</v>
+        <v>46191.782318287034</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F43" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G43" s="9" t="s">
-        <v>161</v>
-      </c>
-      <c r="H43" s="9" t="s">
-        <v>162</v>
-      </c>
-      <c r="I43" s="8">
-        <v>46122</v>
-      </c>
-      <c r="J43" s="8">
-        <v>46125</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H43" s="9"/>
+      <c r="I43" s="9"/>
+      <c r="J43" s="9"/>
       <c r="K43" s="9" t="s">
         <v>26</v>
       </c>
@@ -3760,31 +3750,25 @@
         <v>26</v>
       </c>
       <c r="M43" s="9" t="s">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="N43" s="9" t="s">
-        <v>152</v>
+        <v>26</v>
       </c>
       <c r="O43" s="9" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="P43" s="9" t="s">
-        <v>163</v>
-      </c>
-      <c r="Q43" s="8">
-        <v>46122</v>
-      </c>
-      <c r="R43" s="8">
-        <v>46125</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="Q43" s="9"/>
+      <c r="R43" s="9"/>
       <c r="S43" s="9">
         <v>1</v>
       </c>
-      <c r="T43" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="U43" s="12" t="s">
-        <v>63</v>
+      <c r="T43" s="9"/>
+      <c r="U43" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
@@ -3792,26 +3776,32 @@
         <v>164</v>
       </c>
       <c r="B44" s="5">
-        <v>46079.83218921296</v>
+        <v>46079.83218950231</v>
       </c>
       <c r="C44" s="5">
-        <v>46191.78230420139</v>
+        <v>46191.782240671295</v>
       </c>
       <c r="D44" s="5">
-        <v>46191.782318287034</v>
+        <v>46191.78225513889</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>165</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H44" s="6"/>
-      <c r="I44" s="6"/>
-      <c r="J44" s="6"/>
+        <v>166</v>
+      </c>
+      <c r="H44" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="I44" s="5">
+        <v>46126</v>
+      </c>
+      <c r="J44" s="5">
+        <v>46127</v>
+      </c>
       <c r="K44" s="6" t="s">
         <v>26</v>
       </c>
@@ -3819,57 +3809,63 @@
         <v>26</v>
       </c>
       <c r="M44" s="6" t="s">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>26</v>
+        <v>162</v>
       </c>
       <c r="O44" s="6" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="P44" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q44" s="6"/>
-      <c r="R44" s="6"/>
+        <v>168</v>
+      </c>
+      <c r="Q44" s="5">
+        <v>46126</v>
+      </c>
+      <c r="R44" s="5">
+        <v>46127</v>
+      </c>
       <c r="S44" s="6">
         <v>1</v>
       </c>
-      <c r="T44" s="6"/>
+      <c r="T44" s="10" t="s">
+        <v>31</v>
+      </c>
       <c r="U44" s="11" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="B45" s="8">
+        <v>46079.832189768524</v>
+      </c>
+      <c r="C45" s="8">
+        <v>46191.78228831018</v>
+      </c>
+      <c r="D45" s="8">
+        <v>46191.78230329861</v>
+      </c>
+      <c r="E45" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="F45" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G45" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="H45" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="B45" s="8">
-        <v>46079.83218950231</v>
-      </c>
-      <c r="C45" s="8">
-        <v>46191.782240671295</v>
-      </c>
-      <c r="D45" s="8">
-        <v>46191.78225513889</v>
-      </c>
-      <c r="E45" s="9" t="s">
-        <v>168</v>
-      </c>
-      <c r="F45" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G45" s="9" t="s">
-        <v>169</v>
-      </c>
-      <c r="H45" s="9" t="s">
-        <v>170</v>
-      </c>
       <c r="I45" s="8">
-        <v>46126</v>
+        <v>46128</v>
       </c>
       <c r="J45" s="8">
-        <v>46127</v>
+        <v>46134</v>
       </c>
       <c r="K45" s="9" t="s">
         <v>26</v>
@@ -3881,19 +3877,19 @@
         <v>26</v>
       </c>
       <c r="N45" s="9" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="O45" s="9" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="P45" s="9" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="Q45" s="8">
-        <v>46126</v>
+        <v>46128</v>
       </c>
       <c r="R45" s="8">
-        <v>46127</v>
+        <v>46134</v>
       </c>
       <c r="S45" s="9">
         <v>1</v>
@@ -3907,34 +3903,32 @@
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B46" s="5">
-        <v>46079.832189768524</v>
+        <v>46079.8321887037</v>
       </c>
       <c r="C46" s="5">
-        <v>46191.78228831018</v>
+        <v>46191.78193627315</v>
       </c>
       <c r="D46" s="5">
-        <v>46191.78230329861</v>
+        <v>46191.7823071875</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>169</v>
+        <v>158</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="I46" s="5">
-        <v>46128</v>
-      </c>
+        <v>159</v>
+      </c>
+      <c r="I46" s="6"/>
       <c r="J46" s="5">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="K46" s="6" t="s">
         <v>26</v>
@@ -3946,19 +3940,19 @@
         <v>26</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="P46" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="Q46" s="5">
-        <v>46128</v>
+        <v>46135</v>
       </c>
       <c r="R46" s="5">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="S46" s="6">
         <v>1</v>
@@ -3966,39 +3960,35 @@
       <c r="T46" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U46" s="11" t="s">
-        <v>32</v>
+      <c r="U46" s="12" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B47" s="8">
-        <v>46079.8321887037</v>
+        <v>46079.83218896991</v>
       </c>
       <c r="C47" s="8">
-        <v>46191.78193627315</v>
+        <v>46191.78245119213</v>
       </c>
       <c r="D47" s="8">
-        <v>46191.7823071875</v>
+        <v>46191.782462372685</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>177</v>
+        <v>149</v>
       </c>
       <c r="F47" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>161</v>
-      </c>
-      <c r="H47" s="9" t="s">
-        <v>162</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H47" s="9"/>
       <c r="I47" s="9"/>
-      <c r="J47" s="8">
-        <v>46135</v>
-      </c>
+      <c r="J47" s="9"/>
       <c r="K47" s="9" t="s">
         <v>26</v>
       </c>
@@ -4006,58 +3996,58 @@
         <v>26</v>
       </c>
       <c r="M47" s="9" t="s">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="N47" s="9" t="s">
-        <v>165</v>
+        <v>26</v>
       </c>
       <c r="O47" s="9" t="s">
         <v>178</v>
       </c>
       <c r="P47" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="Q47" s="8">
-        <v>46135</v>
-      </c>
-      <c r="R47" s="8">
-        <v>46135</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="Q47" s="9"/>
+      <c r="R47" s="9"/>
       <c r="S47" s="9">
         <v>1</v>
       </c>
-      <c r="T47" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="U47" s="12" t="s">
-        <v>63</v>
+      <c r="T47" s="9"/>
+      <c r="U47" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B48" s="5">
+        <v>46079.83218923611</v>
+      </c>
+      <c r="C48" s="5">
+        <v>46191.78241675926</v>
+      </c>
+      <c r="D48" s="5">
+        <v>46191.78243247685</v>
+      </c>
+      <c r="E48" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="B48" s="5">
-        <v>46079.83218896991</v>
-      </c>
-      <c r="C48" s="5">
-        <v>46191.78245119213</v>
-      </c>
-      <c r="D48" s="5">
-        <v>46191.782462372685</v>
-      </c>
-      <c r="E48" s="6" t="s">
-        <v>152</v>
-      </c>
       <c r="F48" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H48" s="6"/>
-      <c r="I48" s="6"/>
-      <c r="J48" s="6"/>
+        <v>153</v>
+      </c>
+      <c r="H48" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="I48" s="5">
+        <v>46094</v>
+      </c>
+      <c r="J48" s="5">
+        <v>46097</v>
+      </c>
       <c r="K48" s="6" t="s">
         <v>26</v>
       </c>
@@ -4065,23 +4055,29 @@
         <v>26</v>
       </c>
       <c r="M48" s="6" t="s">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>26</v>
+        <v>149</v>
       </c>
       <c r="O48" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="P48" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="P48" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q48" s="6"/>
-      <c r="R48" s="6"/>
+      <c r="Q48" s="5">
+        <v>46094</v>
+      </c>
+      <c r="R48" s="5">
+        <v>46097</v>
+      </c>
       <c r="S48" s="6">
         <v>1</v>
       </c>
-      <c r="T48" s="6"/>
+      <c r="T48" s="10" t="s">
+        <v>31</v>
+      </c>
       <c r="U48" s="11" t="s">
         <v>32</v>
       </c>
@@ -4091,13 +4087,13 @@
         <v>182</v>
       </c>
       <c r="B49" s="8">
-        <v>46079.83218923611</v>
+        <v>46079.832189513894</v>
       </c>
       <c r="C49" s="8">
-        <v>46191.78241675926</v>
+        <v>46191.78242726852</v>
       </c>
       <c r="D49" s="8">
-        <v>46191.78243247685</v>
+        <v>46191.78244430556</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>183</v>
@@ -4106,16 +4102,16 @@
         <v>26</v>
       </c>
       <c r="G49" s="9" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="H49" s="9" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="I49" s="8">
-        <v>46094</v>
+        <v>46112</v>
       </c>
       <c r="J49" s="8">
-        <v>46097</v>
+        <v>46113</v>
       </c>
       <c r="K49" s="9" t="s">
         <v>26</v>
@@ -4127,19 +4123,19 @@
         <v>26</v>
       </c>
       <c r="N49" s="9" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="O49" s="9" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="P49" s="9" t="s">
         <v>184</v>
       </c>
       <c r="Q49" s="8">
-        <v>46094</v>
+        <v>46112</v>
       </c>
       <c r="R49" s="8">
-        <v>46097</v>
+        <v>46113</v>
       </c>
       <c r="S49" s="9">
         <v>1</v>
@@ -4156,13 +4152,13 @@
         <v>185</v>
       </c>
       <c r="B50" s="5">
-        <v>46079.832189513894</v>
+        <v>46079.83218978009</v>
       </c>
       <c r="C50" s="5">
-        <v>46191.78242726852</v>
+        <v>46191.782435497684</v>
       </c>
       <c r="D50" s="5">
-        <v>46191.78244430556</v>
+        <v>46191.78245195602</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>186</v>
@@ -4171,16 +4167,16 @@
         <v>26</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="I50" s="5">
-        <v>46112</v>
+        <v>46127</v>
       </c>
       <c r="J50" s="5">
-        <v>46113</v>
+        <v>46128</v>
       </c>
       <c r="K50" s="6" t="s">
         <v>26</v>
@@ -4192,19 +4188,19 @@
         <v>26</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="O50" s="6" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="P50" s="6" t="s">
         <v>187</v>
       </c>
       <c r="Q50" s="5">
-        <v>46112</v>
+        <v>46127</v>
       </c>
       <c r="R50" s="5">
-        <v>46113</v>
+        <v>46128</v>
       </c>
       <c r="S50" s="6">
         <v>1</v>
@@ -4221,32 +4217,24 @@
         <v>188</v>
       </c>
       <c r="B51" s="8">
-        <v>46079.83218978009</v>
-      </c>
-      <c r="C51" s="8">
-        <v>46191.782435497684</v>
-      </c>
+        <v>46079.8321903125</v>
+      </c>
+      <c r="C51" s="9"/>
       <c r="D51" s="8">
-        <v>46191.78245195602</v>
+        <v>46191.78261115741</v>
       </c>
       <c r="E51" s="9" t="s">
         <v>189</v>
       </c>
       <c r="F51" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G51" s="9" t="s">
-        <v>156</v>
-      </c>
-      <c r="H51" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="I51" s="8">
-        <v>46127</v>
-      </c>
-      <c r="J51" s="8">
-        <v>46128</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H51" s="9"/>
+      <c r="I51" s="9"/>
+      <c r="J51" s="9"/>
       <c r="K51" s="9" t="s">
         <v>26</v>
       </c>
@@ -4254,31 +4242,23 @@
         <v>26</v>
       </c>
       <c r="M51" s="9" t="s">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="N51" s="9" t="s">
-        <v>152</v>
+        <v>26</v>
       </c>
       <c r="O51" s="9" t="s">
-        <v>114</v>
+        <v>190</v>
       </c>
       <c r="P51" s="9" t="s">
-        <v>190</v>
-      </c>
-      <c r="Q51" s="8">
-        <v>46127</v>
-      </c>
-      <c r="R51" s="8">
-        <v>46128</v>
-      </c>
-      <c r="S51" s="9">
-        <v>1</v>
-      </c>
-      <c r="T51" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="U51" s="11" t="s">
-        <v>32</v>
+        <v>26</v>
+      </c>
+      <c r="Q51" s="9"/>
+      <c r="R51" s="9"/>
+      <c r="S51" s="9"/>
+      <c r="T51" s="9"/>
+      <c r="U51" s="12" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
@@ -4286,24 +4266,32 @@
         <v>191</v>
       </c>
       <c r="B52" s="5">
-        <v>46079.8321903125</v>
-      </c>
-      <c r="C52" s="6"/>
+        <v>46079.83219059028</v>
+      </c>
+      <c r="C52" s="5">
+        <v>46191.78238421296</v>
+      </c>
       <c r="D52" s="5">
-        <v>46191.78261115741</v>
+        <v>46191.7824008912</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>192</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H52" s="6"/>
-      <c r="I52" s="6"/>
-      <c r="J52" s="6"/>
+        <v>72</v>
+      </c>
+      <c r="H52" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="I52" s="5">
+        <v>46136</v>
+      </c>
+      <c r="J52" s="5">
+        <v>46142</v>
+      </c>
       <c r="K52" s="6" t="s">
         <v>26</v>
       </c>
@@ -4311,55 +4299,63 @@
         <v>26</v>
       </c>
       <c r="M52" s="6" t="s">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>26</v>
+        <v>189</v>
       </c>
       <c r="O52" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="P52" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="P52" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q52" s="6"/>
-      <c r="R52" s="6"/>
-      <c r="S52" s="6"/>
-      <c r="T52" s="6"/>
-      <c r="U52" s="12" t="s">
-        <v>63</v>
+      <c r="Q52" s="5">
+        <v>46136</v>
+      </c>
+      <c r="R52" s="5">
+        <v>46142</v>
+      </c>
+      <c r="S52" s="6">
+        <v>1</v>
+      </c>
+      <c r="T52" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="U52" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B53" s="8">
-        <v>46079.83219059028</v>
+        <v>46079.832187673615</v>
       </c>
       <c r="C53" s="8">
-        <v>46191.78238421296</v>
+        <v>46191.7824912037</v>
       </c>
       <c r="D53" s="8">
-        <v>46191.7824008912</v>
+        <v>46191.78250809028</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G53" s="9" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="H53" s="9" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I53" s="8">
-        <v>46136</v>
+        <v>46146</v>
       </c>
       <c r="J53" s="8">
-        <v>46142</v>
+        <v>46146</v>
       </c>
       <c r="K53" s="9" t="s">
         <v>26</v>
@@ -4371,25 +4367,25 @@
         <v>26</v>
       </c>
       <c r="N53" s="9" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="O53" s="9" t="s">
-        <v>177</v>
+        <v>197</v>
       </c>
       <c r="P53" s="9" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="Q53" s="8">
-        <v>46136</v>
+        <v>46146</v>
       </c>
       <c r="R53" s="8">
-        <v>46142</v>
+        <v>46146</v>
       </c>
       <c r="S53" s="9">
         <v>1</v>
       </c>
       <c r="T53" s="12" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="U53" s="11" t="s">
         <v>32</v>
@@ -4397,64 +4393,64 @@
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B54" s="5">
+        <v>46079.832188009255</v>
+      </c>
+      <c r="C54" s="5">
+        <v>46191.78258708333</v>
+      </c>
+      <c r="D54" s="5">
+        <v>46191.78260511574</v>
+      </c>
+      <c r="E54" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="F54" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G54" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="H54" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="I54" s="5">
+        <v>46147</v>
+      </c>
+      <c r="J54" s="5">
+        <v>46147</v>
+      </c>
+      <c r="K54" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L54" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M54" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N54" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="O54" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="P54" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="B54" s="5">
-        <v>46079.832187673615</v>
-      </c>
-      <c r="C54" s="5">
-        <v>46191.7824912037</v>
-      </c>
-      <c r="D54" s="5">
-        <v>46191.78250809028</v>
-      </c>
-      <c r="E54" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="F54" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G54" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="H54" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="I54" s="5">
-        <v>46146</v>
-      </c>
-      <c r="J54" s="5">
-        <v>46146</v>
-      </c>
-      <c r="K54" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L54" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M54" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N54" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="O54" s="6" t="s">
-        <v>200</v>
-      </c>
-      <c r="P54" s="6" t="s">
-        <v>201</v>
-      </c>
       <c r="Q54" s="5">
-        <v>46146</v>
+        <v>46147</v>
       </c>
       <c r="R54" s="5">
-        <v>46146</v>
+        <v>46147</v>
       </c>
       <c r="S54" s="6">
         <v>1</v>
       </c>
-      <c r="T54" s="12" t="s">
-        <v>197</v>
+      <c r="T54" s="11" t="s">
+        <v>90</v>
       </c>
       <c r="U54" s="11" t="s">
         <v>32</v>
@@ -4465,13 +4461,13 @@
         <v>202</v>
       </c>
       <c r="B55" s="8">
-        <v>46079.832188009255</v>
+        <v>46079.83218829861</v>
       </c>
       <c r="C55" s="8">
-        <v>46191.78258708333</v>
+        <v>46191.7825933912</v>
       </c>
       <c r="D55" s="8">
-        <v>46191.78260511574</v>
+        <v>46191.782608622685</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>203</v>
@@ -4480,16 +4476,16 @@
         <v>26</v>
       </c>
       <c r="G55" s="9" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="H55" s="9" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I55" s="8">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="J55" s="8">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="K55" s="9" t="s">
         <v>26</v>
@@ -4501,25 +4497,25 @@
         <v>26</v>
       </c>
       <c r="N55" s="9" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="O55" s="9" t="s">
         <v>204</v>
       </c>
       <c r="P55" s="9" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="Q55" s="8">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="R55" s="8">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="S55" s="9">
         <v>1</v>
       </c>
       <c r="T55" s="11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="U55" s="11" t="s">
         <v>32</v>
@@ -4530,94 +4526,90 @@
         <v>205</v>
       </c>
       <c r="B56" s="5">
-        <v>46079.83218829861</v>
-      </c>
-      <c r="C56" s="5">
-        <v>46191.7825933912</v>
-      </c>
+        <v>46079.83218858796</v>
+      </c>
+      <c r="C56" s="6"/>
       <c r="D56" s="5">
-        <v>46191.782608622685</v>
+        <v>46191.78261061343</v>
       </c>
       <c r="E56" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="F56" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G56" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="H56" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="I56" s="5">
+        <v>46149</v>
+      </c>
+      <c r="J56" s="5">
+        <v>46149</v>
+      </c>
+      <c r="K56" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L56" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M56" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N56" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="O56" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="F56" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G56" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="H56" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="I56" s="5">
-        <v>46148</v>
-      </c>
-      <c r="J56" s="5">
-        <v>46148</v>
-      </c>
-      <c r="K56" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L56" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M56" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N56" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="O56" s="6" t="s">
-        <v>207</v>
-      </c>
       <c r="P56" s="6" t="s">
-        <v>201</v>
+        <v>143</v>
       </c>
       <c r="Q56" s="5">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="R56" s="5">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="S56" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T56" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="U56" s="11" t="s">
-        <v>32</v>
+        <v>90</v>
+      </c>
+      <c r="U56" s="12" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B57" s="8">
-        <v>46079.83218858796</v>
+        <v>46079.83218885417</v>
       </c>
       <c r="C57" s="9"/>
       <c r="D57" s="8">
-        <v>46191.78261061343</v>
+        <v>46153.16820564815</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>149</v>
+        <v>208</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G57" s="9" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="H57" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="I57" s="8">
-        <v>46149</v>
-      </c>
+        <v>72</v>
+      </c>
+      <c r="I57" s="9"/>
       <c r="J57" s="8">
-        <v>46149</v>
+        <v>46153</v>
       </c>
       <c r="K57" s="9" t="s">
         <v>26</v>
@@ -4629,28 +4621,28 @@
         <v>26</v>
       </c>
       <c r="N57" s="9" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="O57" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="P57" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="P57" s="9" t="s">
-        <v>146</v>
-      </c>
       <c r="Q57" s="8">
-        <v>46149</v>
+        <v>46153</v>
       </c>
       <c r="R57" s="8">
-        <v>46149</v>
+        <v>46153</v>
       </c>
       <c r="S57" s="9">
         <v>0</v>
       </c>
       <c r="T57" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="U57" s="12" t="s">
-        <v>63</v>
+        <v>90</v>
+      </c>
+      <c r="U57" s="10" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
@@ -4658,28 +4650,24 @@
         <v>210</v>
       </c>
       <c r="B58" s="5">
-        <v>46079.83218885417</v>
+        <v>46079.83218913194</v>
       </c>
       <c r="C58" s="6"/>
       <c r="D58" s="5">
-        <v>46153.16820564815</v>
+        <v>46087.781215358795</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>211</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="H58" s="6" t="s">
-        <v>75</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H58" s="6"/>
       <c r="I58" s="6"/>
-      <c r="J58" s="5">
-        <v>46153</v>
-      </c>
+      <c r="J58" s="6"/>
       <c r="K58" s="6" t="s">
         <v>26</v>
       </c>
@@ -4687,106 +4675,112 @@
         <v>26</v>
       </c>
       <c r="M58" s="6" t="s">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>192</v>
+        <v>26</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>146</v>
+        <v>212</v>
       </c>
       <c r="P58" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="Q58" s="5">
-        <v>46153</v>
-      </c>
-      <c r="R58" s="5">
-        <v>46153</v>
-      </c>
-      <c r="S58" s="6">
-        <v>0</v>
-      </c>
-      <c r="T58" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="U58" s="10" t="s">
-        <v>94</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="Q58" s="6"/>
+      <c r="R58" s="6"/>
+      <c r="S58" s="6"/>
+      <c r="T58" s="6"/>
+      <c r="U58" s="6"/>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
         <v>213</v>
       </c>
       <c r="B59" s="8">
-        <v>46079.83218913194</v>
+        <v>46079.83218939815</v>
       </c>
       <c r="C59" s="9"/>
       <c r="D59" s="8">
-        <v>46087.781215358795</v>
+        <v>46154.167939374995</v>
       </c>
       <c r="E59" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="F59" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G59" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="H59" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="I59" s="9"/>
+      <c r="J59" s="8">
+        <v>46154</v>
+      </c>
+      <c r="K59" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L59" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M59" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="N59" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="O59" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="P59" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="F59" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="G59" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H59" s="9"/>
-      <c r="I59" s="9"/>
-      <c r="J59" s="9"/>
-      <c r="K59" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L59" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M59" s="9" t="s">
+      <c r="Q59" s="8">
+        <v>46154</v>
+      </c>
+      <c r="R59" s="8">
+        <v>46154</v>
+      </c>
+      <c r="S59" s="9">
         <v>0</v>
       </c>
-      <c r="N59" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="O59" s="9" t="s">
-        <v>215</v>
-      </c>
-      <c r="P59" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q59" s="9"/>
-      <c r="R59" s="9"/>
-      <c r="S59" s="9"/>
-      <c r="T59" s="9"/>
-      <c r="U59" s="9"/>
+      <c r="T59" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="U59" s="10" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B60" s="5">
-        <v>46079.83218939815</v>
+        <v>46079.83218965278</v>
       </c>
       <c r="C60" s="6"/>
       <c r="D60" s="5">
-        <v>46154.167939374995</v>
+        <v>46155.25042148148</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="F60" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G60" s="6" t="s">
-        <v>35</v>
+        <v>72</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="I60" s="6"/>
+        <v>72</v>
+      </c>
+      <c r="I60" s="5">
+        <v>46155</v>
+      </c>
       <c r="J60" s="5">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="K60" s="6" t="s">
         <v>26</v>
@@ -4798,28 +4792,28 @@
         <v>26</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="O60" s="6" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="P60" s="6" t="s">
         <v>217</v>
       </c>
       <c r="Q60" s="5">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="R60" s="5">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="S60" s="6">
         <v>0</v>
       </c>
       <c r="T60" s="11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="U60" s="10" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
@@ -4827,11 +4821,11 @@
         <v>218</v>
       </c>
       <c r="B61" s="8">
-        <v>46079.83218965278</v>
+        <v>46079.83218994213</v>
       </c>
       <c r="C61" s="9"/>
       <c r="D61" s="8">
-        <v>46155.25042148148</v>
+        <v>46156.25043703704</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>219</v>
@@ -4840,16 +4834,14 @@
         <v>26</v>
       </c>
       <c r="G61" s="9" t="s">
-        <v>75</v>
+        <v>166</v>
       </c>
       <c r="H61" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="I61" s="8">
-        <v>46155</v>
-      </c>
+        <v>167</v>
+      </c>
+      <c r="I61" s="9"/>
       <c r="J61" s="8">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="K61" s="9" t="s">
         <v>26</v>
@@ -4861,10 +4853,10 @@
         <v>26</v>
       </c>
       <c r="N61" s="9" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="O61" s="9" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="P61" s="9" t="s">
         <v>220</v>
@@ -4879,10 +4871,10 @@
         <v>0</v>
       </c>
       <c r="T61" s="11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="U61" s="10" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
@@ -4890,11 +4882,11 @@
         <v>221</v>
       </c>
       <c r="B62" s="5">
-        <v>46079.83218994213</v>
+        <v>46079.83219021991</v>
       </c>
       <c r="C62" s="6"/>
       <c r="D62" s="5">
-        <v>46156.25043703704</v>
+        <v>46157.250577071754</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>222</v>
@@ -4903,14 +4895,16 @@
         <v>26</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="I62" s="6"/>
+        <v>167</v>
+      </c>
+      <c r="I62" s="5">
+        <v>46157</v>
+      </c>
       <c r="J62" s="5">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="K62" s="6" t="s">
         <v>26</v>
@@ -4922,7 +4916,7 @@
         <v>26</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="O62" s="6" t="s">
         <v>219</v>
@@ -4931,19 +4925,19 @@
         <v>223</v>
       </c>
       <c r="Q62" s="5">
-        <v>46155</v>
+        <v>46157</v>
       </c>
       <c r="R62" s="5">
-        <v>46155</v>
+        <v>46157</v>
       </c>
       <c r="S62" s="6">
         <v>0</v>
       </c>
       <c r="T62" s="11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="U62" s="10" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
@@ -4951,30 +4945,24 @@
         <v>224</v>
       </c>
       <c r="B63" s="8">
-        <v>46079.83219021991</v>
+        <v>46079.83218761574</v>
       </c>
       <c r="C63" s="9"/>
       <c r="D63" s="8">
-        <v>46157.250577071754</v>
+        <v>46087.78121486111</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>225</v>
       </c>
       <c r="F63" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G63" s="9" t="s">
-        <v>169</v>
-      </c>
-      <c r="H63" s="9" t="s">
-        <v>170</v>
-      </c>
-      <c r="I63" s="8">
-        <v>46157</v>
-      </c>
-      <c r="J63" s="8">
-        <v>46157</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H63" s="9"/>
+      <c r="I63" s="9"/>
+      <c r="J63" s="9"/>
       <c r="K63" s="9" t="s">
         <v>26</v>
       </c>
@@ -4982,56 +4970,52 @@
         <v>26</v>
       </c>
       <c r="M63" s="9" t="s">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="N63" s="9" t="s">
-        <v>214</v>
+        <v>26</v>
       </c>
       <c r="O63" s="9" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="P63" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="Q63" s="8">
-        <v>46157</v>
-      </c>
-      <c r="R63" s="8">
-        <v>46157</v>
-      </c>
-      <c r="S63" s="9">
-        <v>0</v>
-      </c>
-      <c r="T63" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="U63" s="10" t="s">
-        <v>94</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="Q63" s="9"/>
+      <c r="R63" s="9"/>
+      <c r="S63" s="9"/>
+      <c r="T63" s="9"/>
+      <c r="U63" s="9"/>
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
         <v>227</v>
       </c>
       <c r="B64" s="5">
-        <v>46079.83218761574</v>
+        <v>46079.832188368055</v>
       </c>
       <c r="C64" s="6"/>
       <c r="D64" s="5">
-        <v>46087.78121486111</v>
+        <v>46192.680783738426</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>228</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H64" s="6"/>
-      <c r="I64" s="6"/>
-      <c r="J64" s="6"/>
+        <v>229</v>
+      </c>
+      <c r="H64" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="I64" s="5">
+        <v>46160</v>
+      </c>
+      <c r="J64" s="5">
+        <v>46168</v>
+      </c>
       <c r="K64" s="6" t="s">
         <v>26</v>
       </c>
@@ -5039,45 +5023,55 @@
         <v>26</v>
       </c>
       <c r="M64" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N64" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="O64" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="P64" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="Q64" s="5">
+        <v>46160</v>
+      </c>
+      <c r="R64" s="5">
+        <v>46168</v>
+      </c>
+      <c r="S64" s="6">
         <v>0</v>
       </c>
-      <c r="N64" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="O64" s="6" t="s">
-        <v>229</v>
-      </c>
-      <c r="P64" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q64" s="6"/>
-      <c r="R64" s="6"/>
-      <c r="S64" s="6"/>
-      <c r="T64" s="6"/>
-      <c r="U64" s="6"/>
+      <c r="T64" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="U64" s="10" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B65" s="8">
-        <v>46079.832188368055</v>
+        <v>46079.832188009255</v>
       </c>
       <c r="C65" s="9"/>
       <c r="D65" s="8">
-        <v>46169.18880791667</v>
+        <v>46169.188807025464</v>
       </c>
       <c r="E65" s="9" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F65" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G65" s="9" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="H65" s="9" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="I65" s="8">
         <v>46160</v>
@@ -5095,13 +5089,13 @@
         <v>26</v>
       </c>
       <c r="N65" s="9" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="O65" s="9" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="P65" s="9" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="Q65" s="8">
         <v>46160</v>
@@ -5116,70 +5110,7 @@
         <v>31</v>
       </c>
       <c r="U65" s="10" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="66" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A66" s="4" t="s">
-        <v>235</v>
-      </c>
-      <c r="B66" s="5">
-        <v>46079.832188009255</v>
-      </c>
-      <c r="C66" s="6"/>
-      <c r="D66" s="5">
-        <v>46169.188807025464</v>
-      </c>
-      <c r="E66" s="6" t="s">
-        <v>236</v>
-      </c>
-      <c r="F66" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G66" s="6" t="s">
-        <v>232</v>
-      </c>
-      <c r="H66" s="6" t="s">
-        <v>233</v>
-      </c>
-      <c r="I66" s="5">
-        <v>46160</v>
-      </c>
-      <c r="J66" s="5">
-        <v>46168</v>
-      </c>
-      <c r="K66" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L66" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M66" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N66" s="6" t="s">
-        <v>228</v>
-      </c>
-      <c r="O66" s="6" t="s">
-        <v>225</v>
-      </c>
-      <c r="P66" s="6" t="s">
-        <v>228</v>
-      </c>
-      <c r="Q66" s="5">
-        <v>46160</v>
-      </c>
-      <c r="R66" s="5">
-        <v>46168</v>
-      </c>
-      <c r="S66" s="6">
-        <v>0</v>
-      </c>
-      <c r="T66" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="U66" s="10" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>